<commit_message>
Refresh palette review sheet after second round of tweaks
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TYXBizXkFLZPNyuxdiHepz
</commit_message>
<xml_diff>
--- a/sam_themes_palette_review.xlsx
+++ b/sam_themes_palette_review.xlsx
@@ -275,12 +275,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C17858"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00341524"/>
+        <fgColor rgb="00D2A24A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00350D1E"/>
       </patternFill>
     </fill>
     <fill>
@@ -385,12 +385,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C98868"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001E2418"/>
+        <fgColor rgb="003F7A52"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002A1810"/>
       </patternFill>
     </fill>
     <fill>
@@ -682,7 +682,7 @@
     <xf numFmtId="0" fontId="8" fillId="39" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="40" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="40" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="41" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -748,7 +748,7 @@
     <xf numFmtId="0" fontId="8" fillId="61" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="62" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="62" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="63" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1649,7 +1649,7 @@
       <c r="E13" s="7" t="inlineStr">
         <is>
           <t>镜绯红
-Rouge Lens</t>
+Crimson Lens</t>
         </is>
       </c>
       <c r="F13" s="27" t="inlineStr">
@@ -1765,8 +1765,8 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>银灰猫眼
-Mauve Fox</t>
+          <t>紫雾榛眸
+Hazel Mauve</t>
         </is>
       </c>
       <c r="F16" s="33" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>黑貂皮大氅
+          <t>貂皮大氅黑
 Mink Black</t>
         </is>
       </c>
@@ -1994,24 +1994,24 @@
       </c>
       <c r="D22" s="44" t="inlineStr">
         <is>
-          <t>#C17858</t>
+          <t>#D2A24A</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>铜锈玫瑰
-Copper Rose</t>
+          <t>殖民地铜金
+Colonial Gilt</t>
         </is>
       </c>
       <c r="F22" s="45" t="inlineStr">
         <is>
-          <t>#341524</t>
+          <t>#350D1E</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>绒夜玫红
-Rose Velvet Night</t>
+          <t>海报品红夜
+Poster Magenta Night</t>
         </is>
       </c>
       <c r="H22" s="9" t="inlineStr"/>
@@ -2049,7 +2049,7 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>星尘墨夜
+          <t>苍穹墨夜
 Stardust Night</t>
         </is>
       </c>
@@ -2272,8 +2272,8 @@
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>方块烈焰
-Diamond Blaze</t>
+          <t>方块J焰
+Jack of Diamonds</t>
         </is>
       </c>
       <c r="F29" s="59" t="inlineStr">
@@ -2423,24 +2423,24 @@
       </c>
       <c r="D33" s="66" t="inlineStr">
         <is>
-          <t>#C98868</t>
+          <t>#3F7A52</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>陶土暖橘
-Terracotta Warm</t>
+          <t>敞篷车绿
+Racing Green</t>
         </is>
       </c>
       <c r="F33" s="67" t="inlineStr">
         <is>
-          <t>#1E2418</t>
+          <t>#2A1810</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>退伍橄榄
-Old Olive</t>
+          <t>别墅夏夜
+Villa Summer Night</t>
         </is>
       </c>
       <c r="H33" s="9" t="inlineStr"/>
@@ -2974,8 +2974,8 @@
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>枪管冷银光
-Gunmetal Silver</t>
+          <t>冷银弹壳光
+Casing Silver</t>
         </is>
       </c>
       <c r="F47" s="94" t="inlineStr">

</xml_diff>